<commit_message>
fix: upload & manual entry
</commit_message>
<xml_diff>
--- a/uploads/Transaction_Template.xlsx
+++ b/uploads/Transaction_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Connie Ramirez\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{237D7966-4BED-40A0-9069-19526B5197B5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4D2810D-6FA1-406F-865E-8753295BCB01}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="15200" windowHeight="6810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="42">
   <si>
     <t>#</t>
   </si>
@@ -119,27 +119,9 @@
     <t>Rent Expense</t>
   </si>
   <si>
-    <t>Purchase of Office Supplies</t>
-  </si>
-  <si>
-    <t>Office Supplies</t>
-  </si>
-  <si>
-    <t>Client Consultation Payment</t>
-  </si>
-  <si>
-    <t>Service Revenue</t>
-  </si>
-  <si>
     <t>Gcash</t>
   </si>
   <si>
-    <t>Purchase of Inventory (Raw Materials)</t>
-  </si>
-  <si>
-    <t>Cost of Goods Sold</t>
-  </si>
-  <si>
     <t>Store Water Utility Bill</t>
   </si>
   <si>
@@ -156,15 +138,6 @@
   </si>
   <si>
     <t>OR-8992</t>
-  </si>
-  <si>
-    <t>OR-5104</t>
-  </si>
-  <si>
-    <t>OR-0002</t>
-  </si>
-  <si>
-    <t>OR-3105</t>
   </si>
   <si>
     <t>OR-7882</t>
@@ -514,7 +487,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="12.90625" customWidth="1"/>
@@ -575,7 +548,7 @@
         <v>9</v>
       </c>
       <c r="H2" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
@@ -601,7 +574,7 @@
         <v>15</v>
       </c>
       <c r="H3" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -609,25 +582,25 @@
         <v>3</v>
       </c>
       <c r="B4" s="1">
-        <v>46206</v>
+        <v>46213</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
         <v>18</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F4">
-        <v>1250.5</v>
+        <v>850</v>
       </c>
       <c r="G4" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="H4" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -635,25 +608,25 @@
         <v>4</v>
       </c>
       <c r="B5" s="1">
-        <v>46208</v>
+        <v>46215</v>
       </c>
       <c r="C5" t="s">
         <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E5" t="s">
         <v>35</v>
       </c>
       <c r="F5">
-        <v>4500</v>
+        <v>75000</v>
       </c>
       <c r="G5" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="H5" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -661,103 +634,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="1">
-        <v>46209</v>
+        <v>46218</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E6" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="F6">
-        <v>6200</v>
+        <v>3200</v>
       </c>
       <c r="G6" t="s">
         <v>9</v>
       </c>
       <c r="H6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" s="1">
-        <v>46213</v>
-      </c>
-      <c r="C7" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7">
-        <v>850</v>
-      </c>
-      <c r="G7" t="s">
-        <v>36</v>
-      </c>
-      <c r="H7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" s="1">
-        <v>46215</v>
-      </c>
-      <c r="C8" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" t="s">
         <v>41</v>
-      </c>
-      <c r="F8">
-        <v>75000</v>
-      </c>
-      <c r="G8" t="s">
-        <v>36</v>
-      </c>
-      <c r="H8" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" s="1">
-        <v>46218</v>
-      </c>
-      <c r="C9" t="s">
-        <v>42</v>
-      </c>
-      <c r="D9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F9">
-        <v>3200</v>
-      </c>
-      <c r="G9" t="s">
-        <v>9</v>
-      </c>
-      <c r="H9" t="s">
-        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -770,19 +665,19 @@
           <x14:formula1>
             <xm:f>Lists!$A$1:$A$5</xm:f>
           </x14:formula1>
-          <xm:sqref>D2 D3 D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D45 D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 D74 D75 D76 D77 D78 D79 D80 D81 D82 D83 D84 D85 D86 D87 D88 D89 D90 D91 D92 D93 D94 D95 D96 D97 D98 D99 D100 D101 D102 D103 D104 D105 D106 D107 D108 D109 D110 D111 D112 D113 D114 D115 D116 D117 D118 D119 D120 D121 D122 D123 D124 D125 D126 D127 D128 D129 D130 D131 D132 D133 D134 D135 D136 D137 D138 D139 D140 D141 D142 D143 D144 D145 D146 D147 D148 D149 D150 D151 D152 D153 D154 D155 D156 D157 D158 D159 D160 D161 D162 D163 D164 D165 D166 D167 D168 D169 D170 D171 D172 D173 D174 D175 D176 D177 D178 D179 D180 D181 D182 D183 D184 D185 D186 D187 D188 D189 D190 D191 D192 D193 D194 D195 D196 D197 D198 D199 D200 D201 D202 D203 D204 D205 D206 D207 D208 D209 D210 D211 D212 D213 D214 D215 D216 D217 D218 D219 D220 D221 D222 D223 D224 D225 D226 D227 D228 D229 D230 D231 D232 D233 D234 D235 D236 D237 D238 D239 D240 D241 D242 D243 D244 D245 D246 D247 D248 D249 D250 D251 D252 D253 D254 D255 D256 D257 D258 D259 D260 D261 D262 D263 D264 D265 D266 D267 D268 D269 D270 D271 D272 D273 D274 D275 D276 D277 D278 D279 D280 D281 D282 D283 D284 D285 D286 D287 D288 D289 D290 D291 D292 D293 D294 D295 D296 D297 D298 D299 D300 D301 D302 D303 D304 D305 D306 D307 D308 D309 D310 D311 D312 D313 D314 D315 D316 D317 D318 D319 D320 D321 D322 D323 D324 D325 D326 D327 D328 D329 D330 D331 D332 D333 D334 D335 D336 D337 D338 D339 D340 D341 D342 D343 D344 D345 D346 D347 D348 D349 D350 D351 D352 D353 D354 D355 D356 D357 D358 D359 D360 D361 D362 D363 D364 D365 D366 D367 D368 D369 D370 D371 D372 D373 D374 D375 D376 D377 D378 D379 D380 D381 D382 D383 D384 D385 D386 D387 D388 D389 D390 D391 D392 D393 D394 D395 D396 D397 D398 D399 D400 D401 D402 D403 D404 D405 D406 D407 D408 D409 D410 D411 D412 D413 D414 D415 D416 D417 D418 D419 D420 D421 D422 D423 D424 D425 D426 D427 D428 D429 D430 D431 D432 D433 D434 D435 D436 D437 D438 D439 D440 D441 D442 D443 D444 D445 D446 D447 D448 D449 D450 D451 D452 D453 D454 D455 D456 D457 D458 D459 D460 D461 D462 D463 D464 D465 D466 D467 D468 D469 D470 D471 D472 D473 D474 D475 D476 D477 D478 D479 D480 D481 D482 D483 D484 D485 D486 D487 D488 D489 D490 D491 D492 D493 D494 D495 D496 D497 D498 D499 D500 D501 D502 D503 D504 D505 D506 D507 D508 D509 D510 D511 D512 D513 D514 D515 D516 D517 D518 D519 D520 D521 D522 D523 D524 D525 D526 D527 D528 D529 D530 D531 D532 D533 D534 D535 D536 D537 D538 D539 D540 D541 D542 D543 D544 D545 D546 D547 D548 D549 D550 D551 D552 D553 D554 D555 D556 D557 D558 D559 D560 D561 D562 D563 D564 D565 D566 D567 D568 D569 D570 D571 D572 D573 D574 D575 D576 D577 D578 D579 D580 D581 D582 D583 D584 D585 D586 D587 D588 D589 D590 D591 D592 D593 D594 D595 D596 D597 D598 D599 D600 D601 D602 D603 D604 D605 D606 D607 D608 D609 D610 D611 D612 D613 D614 D615 D616 D617 D618 D619 D620 D621 D622 D623 D624 D625 D626 D627 D628 D629 D630 D631 D632 D633 D634 D635 D636 D637 D638 D639 D640 D641 D642 D643 D644 D645 D646 D647 D648 D649 D650 D651 D652 D653 D654 D655 D656 D657 D658 D659 D660 D661 D662 D663 D664 D665 D666 D667 D668 D669 D670 D671 D672 D673 D674 D675 D676 D677 D678 D679 D680 D681 D682 D683 D684 D685 D686 D687 D688 D689 D690 D691 D692 D693 D694 D695 D696 D697 D698 D699 D700 D701 D702 D703 D704 D705 D706 D707 D708 D709 D710 D711 D712 D713 D714 D715 D716 D717 D718 D719 D720 D721 D722 D723 D724 D725 D726 D727 D728 D729 D730 D731 D732 D733 D734 D735 D736 D737 D738 D739 D740 D741 D742 D743 D744 D745 D746 D747 D748 D749 D750 D751 D752 D753 D754 D755 D756 D757 D758 D759 D760 D761 D762 D763 D764 D765 D766 D767 D768 D769 D770 D771 D772 D773 D774 D775 D776 D777 D778 D779 D780 D781 D782 D783 D784 D785 D786 D787 D788 D789 D790 D791 D792 D793 D794 D795 D796 D797 D798 D799 D800 D801 D802 D803 D804 D805 D806 D807 D808 D809 D810 D811 D812 D813 D814 D815 D816 D817 D818 D819 D820 D821 D822 D823 D824 D825 D826 D827 D828 D829 D830 D831 D832 D833 D834 D835 D836 D837 D838 D839 D840 D841 D842 D843 D844 D845 D846 D847 D848 D849 D850 D851 D852 D853 D854 D855 D856 D857 D858 D859 D860 D861 D862 D863 D864 D865 D866 D867 D868 D869 D870 D871 D872 D873 D874 D875 D876 D877 D878 D879 D880 D881 D882 D883 D884 D885 D886 D887 D888 D889 D890 D891 D892 D893 D894 D895 D896 D897 D898 D899 D900 D901 D902 D903 D904 D905 D906 D907 D908 D909 D910 D911 D912 D913 D914 D915 D916 D917 D918 D919 D920 D921 D922 D923 D924 D925 D926 D927 D928 D929 D930 D931 D932 D933 D934 D935 D936 D937 D938 D939 D940 D941 D942 D943 D944 D945 D946 D947 D948 D949 D950 D951 D952 D953 D954 D955 D956 D957 D958 D959 D960 D961 D962 D963 D964 D965 D966 D967 D968 D969 D970 D971 D972 D973 D974 D975 D976 D977 D978 D979 D980 D981 D982 D983 D984 D985 D986 D987 D988 D989 D990 D991 D992 D993 D994 D995 D996 D997 D998 D999</xm:sqref>
+          <xm:sqref>D2 D3 D994 D995 D996 D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D45 D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 D74 D75 D76 D77 D78 D79 D80 D81 D82 D83 D84 D85 D86 D87 D88 D89 D90 D91 D92 D93 D94 D95 D96 D97 D98 D99 D100 D101 D102 D103 D104 D105 D106 D107 D108 D109 D110 D111 D112 D113 D114 D115 D116 D117 D118 D119 D120 D121 D122 D123 D124 D125 D126 D127 D128 D129 D130 D131 D132 D133 D134 D135 D136 D137 D138 D139 D140 D141 D142 D143 D144 D145 D146 D147 D148 D149 D150 D151 D152 D153 D154 D155 D156 D157 D158 D159 D160 D161 D162 D163 D164 D165 D166 D167 D168 D169 D170 D171 D172 D173 D174 D175 D176 D177 D178 D179 D180 D181 D182 D183 D184 D185 D186 D187 D188 D189 D190 D191 D192 D193 D194 D195 D196 D197 D198 D199 D200 D201 D202 D203 D204 D205 D206 D207 D208 D209 D210 D211 D212 D213 D214 D215 D216 D217 D218 D219 D220 D221 D222 D223 D224 D225 D226 D227 D228 D229 D230 D231 D232 D233 D234 D235 D236 D237 D238 D239 D240 D241 D242 D243 D244 D245 D246 D247 D248 D249 D250 D251 D252 D253 D254 D255 D256 D257 D258 D259 D260 D261 D262 D263 D264 D265 D266 D267 D268 D269 D270 D271 D272 D273 D274 D275 D276 D277 D278 D279 D280 D281 D282 D283 D284 D285 D286 D287 D288 D289 D290 D291 D292 D293 D294 D295 D296 D297 D298 D299 D300 D301 D302 D303 D304 D305 D306 D307 D308 D309 D310 D311 D312 D313 D314 D315 D316 D317 D318 D319 D320 D321 D322 D323 D324 D325 D326 D327 D328 D329 D330 D331 D332 D333 D334 D335 D336 D337 D338 D339 D340 D341 D342 D343 D344 D345 D346 D347 D348 D349 D350 D351 D352 D353 D354 D355 D356 D357 D358 D359 D360 D361 D362 D363 D364 D365 D366 D367 D368 D369 D370 D371 D372 D373 D374 D375 D376 D377 D378 D379 D380 D381 D382 D383 D384 D385 D386 D387 D388 D389 D390 D391 D392 D393 D394 D395 D396 D397 D398 D399 D400 D401 D402 D403 D404 D405 D406 D407 D408 D409 D410 D411 D412 D413 D414 D415 D416 D417 D418 D419 D420 D421 D422 D423 D424 D425 D426 D427 D428 D429 D430 D431 D432 D433 D434 D435 D436 D437 D438 D439 D440 D441 D442 D443 D444 D445 D446 D447 D448 D449 D450 D451 D452 D453 D454 D455 D456 D457 D458 D459 D460 D461 D462 D463 D464 D465 D466 D467 D468 D469 D470 D471 D472 D473 D474 D475 D476 D477 D478 D479 D480 D481 D482 D483 D484 D485 D486 D487 D488 D489 D490 D491 D492 D493 D494 D495 D496 D497 D498 D499 D500 D501 D502 D503 D504 D505 D506 D507 D508 D509 D510 D511 D512 D513 D514 D515 D516 D517 D518 D519 D520 D521 D522 D523 D524 D525 D526 D527 D528 D529 D530 D531 D532 D533 D534 D535 D536 D537 D538 D539 D540 D541 D542 D543 D544 D545 D546 D547 D548 D549 D550 D551 D552 D553 D554 D555 D556 D557 D558 D559 D560 D561 D562 D563 D564 D565 D566 D567 D568 D569 D570 D571 D572 D573 D574 D575 D576 D577 D578 D579 D580 D581 D582 D583 D584 D585 D586 D587 D588 D589 D590 D591 D592 D593 D594 D595 D596 D597 D598 D599 D600 D601 D602 D603 D604 D605 D606 D607 D608 D609 D610 D611 D612 D613 D614 D615 D616 D617 D618 D619 D620 D621 D622 D623 D624 D625 D626 D627 D628 D629 D630 D631 D632 D633 D634 D635 D636 D637 D638 D639 D640 D641 D642 D643 D644 D645 D646 D647 D648 D649 D650 D651 D652 D653 D654 D655 D656 D657 D658 D659 D660 D661 D662 D663 D664 D665 D666 D667 D668 D669 D670 D671 D672 D673 D674 D675 D676 D677 D678 D679 D680 D681 D682 D683 D684 D685 D686 D687 D688 D689 D690 D691 D692 D693 D694 D695 D696 D697 D698 D699 D700 D701 D702 D703 D704 D705 D706 D707 D708 D709 D710 D711 D712 D713 D714 D715 D716 D717 D718 D719 D720 D721 D722 D723 D724 D725 D726 D727 D728 D729 D730 D731 D732 D733 D734 D735 D736 D737 D738 D739 D740 D741 D742 D743 D744 D745 D746 D747 D748 D749 D750 D751 D752 D753 D754 D755 D756 D757 D758 D759 D760 D761 D762 D763 D764 D765 D766 D767 D768 D769 D770 D771 D772 D773 D774 D775 D776 D777 D778 D779 D780 D781 D782 D783 D784 D785 D786 D787 D788 D789 D790 D791 D792 D793 D794 D795 D796 D797 D798 D799 D800 D801 D802 D803 D804 D805 D806 D807 D808 D809 D810 D811 D812 D813 D814 D815 D816 D817 D818 D819 D820 D821 D822 D823 D824 D825 D826 D827 D828 D829 D830 D831 D832 D833 D834 D835 D836 D837 D838 D839 D840 D841 D842 D843 D844 D845 D846 D847 D848 D849 D850 D851 D852 D853 D854 D855 D856 D857 D858 D859 D860 D861 D862 D863 D864 D865 D866 D867 D868 D869 D870 D871 D872 D873 D874 D875 D876 D877 D878 D879 D880 D881 D882 D883 D884 D885 D886 D887 D888 D889 D890 D891 D892 D893 D894 D895 D896 D897 D898 D899 D900 D901 D902 D903 D904 D905 D906 D907 D908 D909 D910 D911 D912 D913 D914 D915 D916 D917 D918 D919 D920 D921 D922 D923 D924 D925 D926 D927 D928 D929 D930 D931 D932 D933 D934 D935 D936 D937 D938 D939 D940 D941 D942 D943 D944 D945 D946 D947 D948 D949 D950 D951 D952 D953 D954 D955 D956 D957 D958 D959 D960 D961 D962 D963 D964 D965 D966 D967 D968 D969 D970 D971 D972 D973 D974 D975 D976 D977 D978 D979 D980 D981 D982 D983 D984 D985 D986 D987 D988 D989 D990 D991 D992 D993</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0000-000001000000}">
           <x14:formula1>
             <xm:f>Lists!$B$1:$B$13</xm:f>
           </x14:formula1>
-          <xm:sqref>E2 E3 E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E52 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E72 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E96 E97 E98 E99 E100 E101 E102 E103 E104 E105 E106 E107 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E118 E119 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E134 E135 E136 E137 E138 E139 E140 E141 E142 E143 E144 E145 E146 E147 E148 E149 E150 E151 E152 E153 E154 E155 E156 E157 E158 E159 E160 E161 E162 E163 E164 E165 E166 E167 E168 E169 E170 E171 E172 E173 E174 E175 E176 E177 E178 E179 E180 E181 E182 E183 E184 E185 E186 E187 E188 E189 E190 E191 E192 E193 E194 E195 E196 E197 E198 E199 E200 E201 E202 E203 E204 E205 E206 E207 E208 E209 E210 E211 E212 E213 E214 E215 E216 E217 E218 E219 E220 E221 E222 E223 E224 E225 E226 E227 E228 E229 E230 E231 E232 E233 E234 E235 E236 E237 E238 E239 E240 E241 E242 E243 E244 E245 E246 E247 E248 E249 E250 E251 E252 E253 E254 E255 E256 E257 E258 E259 E260 E261 E262 E263 E264 E265 E266 E267 E268 E269 E270 E271 E272 E273 E274 E275 E276 E277 E278 E279 E280 E281 E282 E283 E284 E285 E286 E287 E288 E289 E290 E291 E292 E293 E294 E295 E296 E297 E298 E299 E300 E301 E302 E303 E304 E305 E306 E307 E308 E309 E310 E311 E312 E313 E314 E315 E316 E317 E318 E319 E320 E321 E322 E323 E324 E325 E326 E327 E328 E329 E330 E331 E332 E333 E334 E335 E336 E337 E338 E339 E340 E341 E342 E343 E344 E345 E346 E347 E348 E349 E350 E351 E352 E353 E354 E355 E356 E357 E358 E359 E360 E361 E362 E363 E364 E365 E366 E367 E368 E369 E370 E371 E372 E373 E374 E375 E376 E377 E378 E379 E380 E381 E382 E383 E384 E385 E386 E387 E388 E389 E390 E391 E392 E393 E394 E395 E396 E397 E398 E399 E400 E401 E402 E403 E404 E405 E406 E407 E408 E409 E410 E411 E412 E413 E414 E415 E416 E417 E418 E419 E420 E421 E422 E423 E424 E425 E426 E427 E428 E429 E430 E431 E432 E433 E434 E435 E436 E437 E438 E439 E440 E441 E442 E443 E444 E445 E446 E447 E448 E449 E450 E451 E452 E453 E454 E455 E456 E457 E458 E459 E460 E461 E462 E463 E464 E465 E466 E467 E468 E469 E470 E471 E472 E473 E474 E475 E476 E477 E478 E479 E480 E481 E482 E483 E484 E485 E486 E487 E488 E489 E490 E491 E492 E493 E494 E495 E496 E497 E498 E499 E500 E501 E502 E503 E504 E505 E506 E507 E508 E509 E510 E511 E512 E513 E514 E515 E516 E517 E518 E519 E520 E521 E522 E523 E524 E525 E526 E527 E528 E529 E530 E531 E532 E533 E534 E535 E536 E537 E538 E539 E540 E541 E542 E543 E544 E545 E546 E547 E548 E549 E550 E551 E552 E553 E554 E555 E556 E557 E558 E559 E560 E561 E562 E563 E564 E565 E566 E567 E568 E569 E570 E571 E572 E573 E574 E575 E576 E577 E578 E579 E580 E581 E582 E583 E584 E585 E586 E587 E588 E589 E590 E591 E592 E593 E594 E595 E596 E597 E598 E599 E600 E601 E602 E603 E604 E605 E606 E607 E608 E609 E610 E611 E612 E613 E614 E615 E616 E617 E618 E619 E620 E621 E622 E623 E624 E625 E626 E627 E628 E629 E630 E631 E632 E633 E634 E635 E636 E637 E638 E639 E640 E641 E642 E643 E644 E645 E646 E647 E648 E649 E650 E651 E652 E653 E654 E655 E656 E657 E658 E659 E660 E661 E662 E663 E664 E665 E666 E667 E668 E669 E670 E671 E672 E673 E674 E675 E676 E677 E678 E679 E680 E681 E682 E683 E684 E685 E686 E687 E688 E689 E690 E691 E692 E693 E694 E695 E696 E697 E698 E699 E700 E701 E702 E703 E704 E705 E706 E707 E708 E709 E710 E711 E712 E713 E714 E715 E716 E717 E718 E719 E720 E721 E722 E723 E724 E725 E726 E727 E728 E729 E730 E731 E732 E733 E734 E735 E736 E737 E738 E739 E740 E741 E742 E743 E744 E745 E746 E747 E748 E749 E750 E751 E752 E753 E754 E755 E756 E757 E758 E759 E760 E761 E762 E763 E764 E765 E766 E767 E768 E769 E770 E771 E772 E773 E774 E775 E776 E777 E778 E779 E780 E781 E782 E783 E784 E785 E786 E787 E788 E789 E790 E791 E792 E793 E794 E795 E796 E797 E798 E799 E800 E801 E802 E803 E804 E805 E806 E807 E808 E809 E810 E811 E812 E813 E814 E815 E816 E817 E818 E819 E820 E821 E822 E823 E824 E825 E826 E827 E828 E829 E830 E831 E832 E833 E834 E835 E836 E837 E838 E839 E840 E841 E842 E843 E844 E845 E846 E847 E848 E849 E850 E851 E852 E853 E854 E855 E856 E857 E858 E859 E860 E861 E862 E863 E864 E865 E866 E867 E868 E869 E870 E871 E872 E873 E874 E875 E876 E877 E878 E879 E880 E881 E882 E883 E884 E885 E886 E887 E888 E889 E890 E891 E892 E893 E894 E895 E896 E897 E898 E899 E900 E901 E902 E903 E904 E905 E906 E907 E908 E909 E910 E911 E912 E913 E914 E915 E916 E917 E918 E919 E920 E921 E922 E923 E924 E925 E926 E927 E928 E929 E930 E931 E932 E933 E934 E935 E936 E937 E938 E939 E940 E941 E942 E943 E944 E945 E946 E947 E948 E949 E950 E951 E952 E953 E954 E955 E956 E957 E958 E959 E960 E961 E962 E963 E964 E965 E966 E967 E968 E969 E970 E971 E972 E973 E974 E975 E976 E977 E978 E979 E980 E981 E982 E983 E984 E985 E986 E987 E988 E989 E990 E991 E992 E993 E994 E995 E996 E997 E998 E999</xm:sqref>
+          <xm:sqref>E2 E3 E994 E995 E996 E4 E5 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E32 E33 E34 E35 E36 E37 E38 E39 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E52 E53 E54 E55 E56 E57 E58 E59 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E72 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E96 E97 E98 E99 E100 E101 E102 E103 E104 E105 E106 E107 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E118 E119 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E134 E135 E136 E137 E138 E139 E140 E141 E142 E143 E144 E145 E146 E147 E148 E149 E150 E151 E152 E153 E154 E155 E156 E157 E158 E159 E160 E161 E162 E163 E164 E165 E166 E167 E168 E169 E170 E171 E172 E173 E174 E175 E176 E177 E178 E179 E180 E181 E182 E183 E184 E185 E186 E187 E188 E189 E190 E191 E192 E193 E194 E195 E196 E197 E198 E199 E200 E201 E202 E203 E204 E205 E206 E207 E208 E209 E210 E211 E212 E213 E214 E215 E216 E217 E218 E219 E220 E221 E222 E223 E224 E225 E226 E227 E228 E229 E230 E231 E232 E233 E234 E235 E236 E237 E238 E239 E240 E241 E242 E243 E244 E245 E246 E247 E248 E249 E250 E251 E252 E253 E254 E255 E256 E257 E258 E259 E260 E261 E262 E263 E264 E265 E266 E267 E268 E269 E270 E271 E272 E273 E274 E275 E276 E277 E278 E279 E280 E281 E282 E283 E284 E285 E286 E287 E288 E289 E290 E291 E292 E293 E294 E295 E296 E297 E298 E299 E300 E301 E302 E303 E304 E305 E306 E307 E308 E309 E310 E311 E312 E313 E314 E315 E316 E317 E318 E319 E320 E321 E322 E323 E324 E325 E326 E327 E328 E329 E330 E331 E332 E333 E334 E335 E336 E337 E338 E339 E340 E341 E342 E343 E344 E345 E346 E347 E348 E349 E350 E351 E352 E353 E354 E355 E356 E357 E358 E359 E360 E361 E362 E363 E364 E365 E366 E367 E368 E369 E370 E371 E372 E373 E374 E375 E376 E377 E378 E379 E380 E381 E382 E383 E384 E385 E386 E387 E388 E389 E390 E391 E392 E393 E394 E395 E396 E397 E398 E399 E400 E401 E402 E403 E404 E405 E406 E407 E408 E409 E410 E411 E412 E413 E414 E415 E416 E417 E418 E419 E420 E421 E422 E423 E424 E425 E426 E427 E428 E429 E430 E431 E432 E433 E434 E435 E436 E437 E438 E439 E440 E441 E442 E443 E444 E445 E446 E447 E448 E449 E450 E451 E452 E453 E454 E455 E456 E457 E458 E459 E460 E461 E462 E463 E464 E465 E466 E467 E468 E469 E470 E471 E472 E473 E474 E475 E476 E477 E478 E479 E480 E481 E482 E483 E484 E485 E486 E487 E488 E489 E490 E491 E492 E493 E494 E495 E496 E497 E498 E499 E500 E501 E502 E503 E504 E505 E506 E507 E508 E509 E510 E511 E512 E513 E514 E515 E516 E517 E518 E519 E520 E521 E522 E523 E524 E525 E526 E527 E528 E529 E530 E531 E532 E533 E534 E535 E536 E537 E538 E539 E540 E541 E542 E543 E544 E545 E546 E547 E548 E549 E550 E551 E552 E553 E554 E555 E556 E557 E558 E559 E560 E561 E562 E563 E564 E565 E566 E567 E568 E569 E570 E571 E572 E573 E574 E575 E576 E577 E578 E579 E580 E581 E582 E583 E584 E585 E586 E587 E588 E589 E590 E591 E592 E593 E594 E595 E596 E597 E598 E599 E600 E601 E602 E603 E604 E605 E606 E607 E608 E609 E610 E611 E612 E613 E614 E615 E616 E617 E618 E619 E620 E621 E622 E623 E624 E625 E626 E627 E628 E629 E630 E631 E632 E633 E634 E635 E636 E637 E638 E639 E640 E641 E642 E643 E644 E645 E646 E647 E648 E649 E650 E651 E652 E653 E654 E655 E656 E657 E658 E659 E660 E661 E662 E663 E664 E665 E666 E667 E668 E669 E670 E671 E672 E673 E674 E675 E676 E677 E678 E679 E680 E681 E682 E683 E684 E685 E686 E687 E688 E689 E690 E691 E692 E693 E694 E695 E696 E697 E698 E699 E700 E701 E702 E703 E704 E705 E706 E707 E708 E709 E710 E711 E712 E713 E714 E715 E716 E717 E718 E719 E720 E721 E722 E723 E724 E725 E726 E727 E728 E729 E730 E731 E732 E733 E734 E735 E736 E737 E738 E739 E740 E741 E742 E743 E744 E745 E746 E747 E748 E749 E750 E751 E752 E753 E754 E755 E756 E757 E758 E759 E760 E761 E762 E763 E764 E765 E766 E767 E768 E769 E770 E771 E772 E773 E774 E775 E776 E777 E778 E779 E780 E781 E782 E783 E784 E785 E786 E787 E788 E789 E790 E791 E792 E793 E794 E795 E796 E797 E798 E799 E800 E801 E802 E803 E804 E805 E806 E807 E808 E809 E810 E811 E812 E813 E814 E815 E816 E817 E818 E819 E820 E821 E822 E823 E824 E825 E826 E827 E828 E829 E830 E831 E832 E833 E834 E835 E836 E837 E838 E839 E840 E841 E842 E843 E844 E845 E846 E847 E848 E849 E850 E851 E852 E853 E854 E855 E856 E857 E858 E859 E860 E861 E862 E863 E864 E865 E866 E867 E868 E869 E870 E871 E872 E873 E874 E875 E876 E877 E878 E879 E880 E881 E882 E883 E884 E885 E886 E887 E888 E889 E890 E891 E892 E893 E894 E895 E896 E897 E898 E899 E900 E901 E902 E903 E904 E905 E906 E907 E908 E909 E910 E911 E912 E913 E914 E915 E916 E917 E918 E919 E920 E921 E922 E923 E924 E925 E926 E927 E928 E929 E930 E931 E932 E933 E934 E935 E936 E937 E938 E939 E940 E941 E942 E943 E944 E945 E946 E947 E948 E949 E950 E951 E952 E953 E954 E955 E956 E957 E958 E959 E960 E961 E962 E963 E964 E965 E966 E967 E968 E969 E970 E971 E972 E973 E974 E975 E976 E977 E978 E979 E980 E981 E982 E983 E984 E985 E986 E987 E988 E989 E990 E991 E992 E993</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>Lists!$C$1:$C$3</xm:f>
           </x14:formula1>
-          <xm:sqref>G2 G3 G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44 G45 G46 G47 G48 G49 G50 G51 G52 G53 G54 G55 G56 G57 G58 G59 G60 G61 G62 G63 G64 G65 G66 G67 G68 G69 G70 G71 G72 G73 G74 G75 G76 G77 G78 G79 G80 G81 G82 G83 G84 G85 G86 G87 G88 G89 G90 G91 G92 G93 G94 G95 G96 G97 G98 G99 G100 G101 G102 G103 G104 G105 G106 G107 G108 G109 G110 G111 G112 G113 G114 G115 G116 G117 G118 G119 G120 G121 G122 G123 G124 G125 G126 G127 G128 G129 G130 G131 G132 G133 G134 G135 G136 G137 G138 G139 G140 G141 G142 G143 G144 G145 G146 G147 G148 G149 G150 G151 G152 G153 G154 G155 G156 G157 G158 G159 G160 G161 G162 G163 G164 G165 G166 G167 G168 G169 G170 G171 G172 G173 G174 G175 G176 G177 G178 G179 G180 G181 G182 G183 G184 G185 G186 G187 G188 G189 G190 G191 G192 G193 G194 G195 G196 G197 G198 G199 G200 G201 G202 G203 G204 G205 G206 G207 G208 G209 G210 G211 G212 G213 G214 G215 G216 G217 G218 G219 G220 G221 G222 G223 G224 G225 G226 G227 G228 G229 G230 G231 G232 G233 G234 G235 G236 G237 G238 G239 G240 G241 G242 G243 G244 G245 G246 G247 G248 G249 G250 G251 G252 G253 G254 G255 G256 G257 G258 G259 G260 G261 G262 G263 G264 G265 G266 G267 G268 G269 G270 G271 G272 G273 G274 G275 G276 G277 G278 G279 G280 G281 G282 G283 G284 G285 G286 G287 G288 G289 G290 G291 G292 G293 G294 G295 G296 G297 G298 G299 G300 G301 G302 G303 G304 G305 G306 G307 G308 G309 G310 G311 G312 G313 G314 G315 G316 G317 G318 G319 G320 G321 G322 G323 G324 G325 G326 G327 G328 G329 G330 G331 G332 G333 G334 G335 G336 G337 G338 G339 G340 G341 G342 G343 G344 G345 G346 G347 G348 G349 G350 G351 G352 G353 G354 G355 G356 G357 G358 G359 G360 G361 G362 G363 G364 G365 G366 G367 G368 G369 G370 G371 G372 G373 G374 G375 G376 G377 G378 G379 G380 G381 G382 G383 G384 G385 G386 G387 G388 G389 G390 G391 G392 G393 G394 G395 G396 G397 G398 G399 G400 G401 G402 G403 G404 G405 G406 G407 G408 G409 G410 G411 G412 G413 G414 G415 G416 G417 G418 G419 G420 G421 G422 G423 G424 G425 G426 G427 G428 G429 G430 G431 G432 G433 G434 G435 G436 G437 G438 G439 G440 G441 G442 G443 G444 G445 G446 G447 G448 G449 G450 G451 G452 G453 G454 G455 G456 G457 G458 G459 G460 G461 G462 G463 G464 G465 G466 G467 G468 G469 G470 G471 G472 G473 G474 G475 G476 G477 G478 G479 G480 G481 G482 G483 G484 G485 G486 G487 G488 G489 G490 G491 G492 G493 G494 G495 G496 G497 G498 G499 G500 G501 G502 G503 G504 G505 G506 G507 G508 G509 G510 G511 G512 G513 G514 G515 G516 G517 G518 G519 G520 G521 G522 G523 G524 G525 G526 G527 G528 G529 G530 G531 G532 G533 G534 G535 G536 G537 G538 G539 G540 G541 G542 G543 G544 G545 G546 G547 G548 G549 G550 G551 G552 G553 G554 G555 G556 G557 G558 G559 G560 G561 G562 G563 G564 G565 G566 G567 G568 G569 G570 G571 G572 G573 G574 G575 G576 G577 G578 G579 G580 G581 G582 G583 G584 G585 G586 G587 G588 G589 G590 G591 G592 G593 G594 G595 G596 G597 G598 G599 G600 G601 G602 G603 G604 G605 G606 G607 G608 G609 G610 G611 G612 G613 G614 G615 G616 G617 G618 G619 G620 G621 G622 G623 G624 G625 G626 G627 G628 G629 G630 G631 G632 G633 G634 G635 G636 G637 G638 G639 G640 G641 G642 G643 G644 G645 G646 G647 G648 G649 G650 G651 G652 G653 G654 G655 G656 G657 G658 G659 G660 G661 G662 G663 G664 G665 G666 G667 G668 G669 G670 G671 G672 G673 G674 G675 G676 G677 G678 G679 G680 G681 G682 G683 G684 G685 G686 G687 G688 G689 G690 G691 G692 G693 G694 G695 G696 G697 G698 G699 G700 G701 G702 G703 G704 G705 G706 G707 G708 G709 G710 G711 G712 G713 G714 G715 G716 G717 G718 G719 G720 G721 G722 G723 G724 G725 G726 G727 G728 G729 G730 G731 G732 G733 G734 G735 G736 G737 G738 G739 G740 G741 G742 G743 G744 G745 G746 G747 G748 G749 G750 G751 G752 G753 G754 G755 G756 G757 G758 G759 G760 G761 G762 G763 G764 G765 G766 G767 G768 G769 G770 G771 G772 G773 G774 G775 G776 G777 G778 G779 G780 G781 G782 G783 G784 G785 G786 G787 G788 G789 G790 G791 G792 G793 G794 G795 G796 G797 G798 G799 G800 G801 G802 G803 G804 G805 G806 G807 G808 G809 G810 G811 G812 G813 G814 G815 G816 G817 G818 G819 G820 G821 G822 G823 G824 G825 G826 G827 G828 G829 G830 G831 G832 G833 G834 G835 G836 G837 G838 G839 G840 G841 G842 G843 G844 G845 G846 G847 G848 G849 G850 G851 G852 G853 G854 G855 G856 G857 G858 G859 G860 G861 G862 G863 G864 G865 G866 G867 G868 G869 G870 G871 G872 G873 G874 G875 G876 G877 G878 G879 G880 G881 G882 G883 G884 G885 G886 G887 G888 G889 G890 G891 G892 G893 G894 G895 G896 G897 G898 G899 G900 G901 G902 G903 G904 G905 G906 G907 G908 G909 G910 G911 G912 G913 G914 G915 G916 G917 G918 G919 G920 G921 G922 G923 G924 G925 G926 G927 G928 G929 G930 G931 G932 G933 G934 G935 G936 G937 G938 G939 G940 G941 G942 G943 G944 G945 G946 G947 G948 G949 G950 G951 G952 G953 G954 G955 G956 G957 G958 G959 G960 G961 G962 G963 G964 G965 G966 G967 G968 G969 G970 G971 G972 G973 G974 G975 G976 G977 G978 G979 G980 G981 G982 G983 G984 G985 G986 G987 G988 G989 G990 G991 G992 G993 G994 G995 G996 G997 G998 G999</xm:sqref>
+          <xm:sqref>G2 G3 G994 G995 G996 G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44 G45 G46 G47 G48 G49 G50 G51 G52 G53 G54 G55 G56 G57 G58 G59 G60 G61 G62 G63 G64 G65 G66 G67 G68 G69 G70 G71 G72 G73 G74 G75 G76 G77 G78 G79 G80 G81 G82 G83 G84 G85 G86 G87 G88 G89 G90 G91 G92 G93 G94 G95 G96 G97 G98 G99 G100 G101 G102 G103 G104 G105 G106 G107 G108 G109 G110 G111 G112 G113 G114 G115 G116 G117 G118 G119 G120 G121 G122 G123 G124 G125 G126 G127 G128 G129 G130 G131 G132 G133 G134 G135 G136 G137 G138 G139 G140 G141 G142 G143 G144 G145 G146 G147 G148 G149 G150 G151 G152 G153 G154 G155 G156 G157 G158 G159 G160 G161 G162 G163 G164 G165 G166 G167 G168 G169 G170 G171 G172 G173 G174 G175 G176 G177 G178 G179 G180 G181 G182 G183 G184 G185 G186 G187 G188 G189 G190 G191 G192 G193 G194 G195 G196 G197 G198 G199 G200 G201 G202 G203 G204 G205 G206 G207 G208 G209 G210 G211 G212 G213 G214 G215 G216 G217 G218 G219 G220 G221 G222 G223 G224 G225 G226 G227 G228 G229 G230 G231 G232 G233 G234 G235 G236 G237 G238 G239 G240 G241 G242 G243 G244 G245 G246 G247 G248 G249 G250 G251 G252 G253 G254 G255 G256 G257 G258 G259 G260 G261 G262 G263 G264 G265 G266 G267 G268 G269 G270 G271 G272 G273 G274 G275 G276 G277 G278 G279 G280 G281 G282 G283 G284 G285 G286 G287 G288 G289 G290 G291 G292 G293 G294 G295 G296 G297 G298 G299 G300 G301 G302 G303 G304 G305 G306 G307 G308 G309 G310 G311 G312 G313 G314 G315 G316 G317 G318 G319 G320 G321 G322 G323 G324 G325 G326 G327 G328 G329 G330 G331 G332 G333 G334 G335 G336 G337 G338 G339 G340 G341 G342 G343 G344 G345 G346 G347 G348 G349 G350 G351 G352 G353 G354 G355 G356 G357 G358 G359 G360 G361 G362 G363 G364 G365 G366 G367 G368 G369 G370 G371 G372 G373 G374 G375 G376 G377 G378 G379 G380 G381 G382 G383 G384 G385 G386 G387 G388 G389 G390 G391 G392 G393 G394 G395 G396 G397 G398 G399 G400 G401 G402 G403 G404 G405 G406 G407 G408 G409 G410 G411 G412 G413 G414 G415 G416 G417 G418 G419 G420 G421 G422 G423 G424 G425 G426 G427 G428 G429 G430 G431 G432 G433 G434 G435 G436 G437 G438 G439 G440 G441 G442 G443 G444 G445 G446 G447 G448 G449 G450 G451 G452 G453 G454 G455 G456 G457 G458 G459 G460 G461 G462 G463 G464 G465 G466 G467 G468 G469 G470 G471 G472 G473 G474 G475 G476 G477 G478 G479 G480 G481 G482 G483 G484 G485 G486 G487 G488 G489 G490 G491 G492 G493 G494 G495 G496 G497 G498 G499 G500 G501 G502 G503 G504 G505 G506 G507 G508 G509 G510 G511 G512 G513 G514 G515 G516 G517 G518 G519 G520 G521 G522 G523 G524 G525 G526 G527 G528 G529 G530 G531 G532 G533 G534 G535 G536 G537 G538 G539 G540 G541 G542 G543 G544 G545 G546 G547 G548 G549 G550 G551 G552 G553 G554 G555 G556 G557 G558 G559 G560 G561 G562 G563 G564 G565 G566 G567 G568 G569 G570 G571 G572 G573 G574 G575 G576 G577 G578 G579 G580 G581 G582 G583 G584 G585 G586 G587 G588 G589 G590 G591 G592 G593 G594 G595 G596 G597 G598 G599 G600 G601 G602 G603 G604 G605 G606 G607 G608 G609 G610 G611 G612 G613 G614 G615 G616 G617 G618 G619 G620 G621 G622 G623 G624 G625 G626 G627 G628 G629 G630 G631 G632 G633 G634 G635 G636 G637 G638 G639 G640 G641 G642 G643 G644 G645 G646 G647 G648 G649 G650 G651 G652 G653 G654 G655 G656 G657 G658 G659 G660 G661 G662 G663 G664 G665 G666 G667 G668 G669 G670 G671 G672 G673 G674 G675 G676 G677 G678 G679 G680 G681 G682 G683 G684 G685 G686 G687 G688 G689 G690 G691 G692 G693 G694 G695 G696 G697 G698 G699 G700 G701 G702 G703 G704 G705 G706 G707 G708 G709 G710 G711 G712 G713 G714 G715 G716 G717 G718 G719 G720 G721 G722 G723 G724 G725 G726 G727 G728 G729 G730 G731 G732 G733 G734 G735 G736 G737 G738 G739 G740 G741 G742 G743 G744 G745 G746 G747 G748 G749 G750 G751 G752 G753 G754 G755 G756 G757 G758 G759 G760 G761 G762 G763 G764 G765 G766 G767 G768 G769 G770 G771 G772 G773 G774 G775 G776 G777 G778 G779 G780 G781 G782 G783 G784 G785 G786 G787 G788 G789 G790 G791 G792 G793 G794 G795 G796 G797 G798 G799 G800 G801 G802 G803 G804 G805 G806 G807 G808 G809 G810 G811 G812 G813 G814 G815 G816 G817 G818 G819 G820 G821 G822 G823 G824 G825 G826 G827 G828 G829 G830 G831 G832 G833 G834 G835 G836 G837 G838 G839 G840 G841 G842 G843 G844 G845 G846 G847 G848 G849 G850 G851 G852 G853 G854 G855 G856 G857 G858 G859 G860 G861 G862 G863 G864 G865 G866 G867 G868 G869 G870 G871 G872 G873 G874 G875 G876 G877 G878 G879 G880 G881 G882 G883 G884 G885 G886 G887 G888 G889 G890 G891 G892 G893 G894 G895 G896 G897 G898 G899 G900 G901 G902 G903 G904 G905 G906 G907 G908 G909 G910 G911 G912 G913 G914 G915 G916 G917 G918 G919 G920 G921 G922 G923 G924 G925 G926 G927 G928 G929 G930 G931 G932 G933 G934 G935 G936 G937 G938 G939 G940 G941 G942 G943 G944 G945 G946 G947 G948 G949 G950 G951 G952 G953 G954 G955 G956 G957 G958 G959 G960 G961 G962 G963 G964 G965 G966 G967 G968 G969 G970 G971 G972 G973 G974 G975 G976 G977 G978 G979 G980 G981 G982 G983 G984 G985 G986 G987 G988 G989 G990 G991 G992 G993</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>